<commit_message>
Update finegray/iivw docs and QA fixtures, remove stale demo console...
</commit_message>
<xml_diff>
--- a/iivw/demo/iivw_reporting_exports.xlsx
+++ b/iivw/demo/iivw_reporting_exports.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="1665">
+  <fonts count="1694">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3308,6 +3308,52 @@
     <font>
       <sz val="10"/>
       <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -5278,6 +5324,28 @@
     </font>
     <font>
       <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -7070,6 +7138,60 @@
     <font>
       <sz val="10"/>
       <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -7357,7 +7479,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1312">
+  <borders count="1341">
     <border>
       <left/>
       <right/>
@@ -11360,6 +11482,83 @@
     </border>
     <border>
       <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="thin"/>
       <top style="none"/>
       <bottom style="medium"/>
@@ -13649,6 +13848,41 @@
     </border>
     <border>
       <left style="none"/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
@@ -16132,6 +16366,97 @@
     </border>
     <border>
       <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="thin"/>
       <top style="none"/>
       <bottom style="medium"/>
@@ -16336,7 +16661,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1312">
+  <cellXfs count="1341">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -18713,394 +19038,394 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="763" fillId="0" borderId="597" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="765" fillId="0" borderId="598" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="767" fillId="0" borderId="599" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="769" fillId="0" borderId="600" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="771" fillId="0" borderId="601" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="773" fillId="0" borderId="602" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="775" fillId="0" borderId="603" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="777" fillId="0" borderId="604" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="779" fillId="0" borderId="605" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="781" fillId="0" borderId="606" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="783" fillId="0" borderId="607" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="785" fillId="0" borderId="608" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="787" fillId="0" borderId="609" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="789" fillId="0" borderId="610" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="791" fillId="0" borderId="611" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="793" fillId="0" borderId="612" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="795" fillId="0" borderId="613" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="797" fillId="0" borderId="614" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="798" fillId="0" borderId="615" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="762" fillId="0" borderId="597" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="763" fillId="0" borderId="598" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="764" fillId="0" borderId="599" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="765" fillId="0" borderId="600" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="766" fillId="0" borderId="601" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="767" fillId="0" borderId="602" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="768" fillId="0" borderId="603" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="769" fillId="0" borderId="604" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="770" fillId="0" borderId="605" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="771" fillId="0" borderId="606" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="772" fillId="0" borderId="607" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="774" fillId="0" borderId="608" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="776" fillId="0" borderId="609" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="778" fillId="0" borderId="610" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="780" fillId="0" borderId="611" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="782" fillId="0" borderId="612" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="784" fillId="0" borderId="613" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="786" fillId="0" borderId="614" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="788" fillId="0" borderId="615" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="790" fillId="0" borderId="616" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="792" fillId="0" borderId="617" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="794" fillId="0" borderId="618" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="796" fillId="0" borderId="619" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="798" fillId="0" borderId="620" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="800" fillId="0" borderId="621" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="802" fillId="0" borderId="622" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="804" fillId="0" borderId="623" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="806" fillId="0" borderId="624" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="808" fillId="0" borderId="625" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="809" fillId="0" borderId="626" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="799" fillId="0" borderId="616" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="810" fillId="0" borderId="627" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="800" fillId="0" borderId="617" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="811" fillId="0" borderId="628" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="801" fillId="0" borderId="618" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="812" fillId="0" borderId="629" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="802" fillId="0" borderId="619" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="813" fillId="0" borderId="630" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="803" fillId="0" borderId="620" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="814" fillId="0" borderId="631" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="804" fillId="0" borderId="621" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="815" fillId="0" borderId="632" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="805" fillId="0" borderId="622" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="816" fillId="0" borderId="633" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="806" fillId="0" borderId="623" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="817" fillId="0" borderId="634" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="807" fillId="0" borderId="624" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="818" fillId="0" borderId="635" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="808" fillId="0" borderId="625" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="819" fillId="0" borderId="636" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="626" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="627" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="628" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="629" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="630" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="631" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="632" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="633" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="634" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="635" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="636" xfId="0"/>
-    <xf numFmtId="0" fontId="810" fillId="0" borderId="637" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="812" fillId="0" borderId="638" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="814" fillId="0" borderId="639" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="816" fillId="0" borderId="640" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="818" fillId="0" borderId="641" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="820" fillId="0" borderId="642" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="822" fillId="0" borderId="643" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="824" fillId="0" borderId="644" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="826" fillId="0" borderId="645" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="828" fillId="0" borderId="646" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="830" fillId="0" borderId="647" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="832" fillId="0" borderId="648" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="834" fillId="0" borderId="649" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="836" fillId="0" borderId="650" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="838" fillId="0" borderId="651" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="840" fillId="0" borderId="652" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="842" fillId="0" borderId="653" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="844" fillId="0" borderId="654" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="846" fillId="0" borderId="655" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="848" fillId="0" borderId="656" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="850" fillId="0" borderId="657" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="852" fillId="0" borderId="658" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="854" fillId="0" borderId="659" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="856" fillId="0" borderId="660" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="858" fillId="0" borderId="661" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="860" fillId="0" borderId="662" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="862" fillId="0" borderId="663" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="864" fillId="0" borderId="664" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="866" fillId="0" borderId="665" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="868" fillId="0" borderId="666" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="870" fillId="0" borderId="667" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="872" fillId="0" borderId="668" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="874" fillId="0" borderId="669" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="876" fillId="0" borderId="670" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="878" fillId="0" borderId="671" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="880" fillId="0" borderId="672" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="882" fillId="0" borderId="673" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="884" fillId="0" borderId="674" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="886" fillId="0" borderId="675" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="888" fillId="0" borderId="676" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="890" fillId="0" borderId="677" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="892" fillId="0" borderId="678" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="894" fillId="0" borderId="679" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="896" fillId="0" borderId="680" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="898" fillId="0" borderId="681" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="900" fillId="0" borderId="682" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="902" fillId="0" borderId="683" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="904" fillId="0" borderId="684" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="906" fillId="0" borderId="685" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="908" fillId="0" borderId="686" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="910" fillId="0" borderId="687" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="912" fillId="0" borderId="688" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="914" fillId="0" borderId="689" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="916" fillId="0" borderId="690" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="918" fillId="0" borderId="691" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="920" fillId="0" borderId="692" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="921" fillId="0" borderId="693" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="922" fillId="0" borderId="694" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="923" fillId="0" borderId="695" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="924" fillId="0" borderId="696" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="925" fillId="0" borderId="697" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="926" fillId="0" borderId="698" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="927" fillId="0" borderId="699" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="928" fillId="0" borderId="700" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="929" fillId="0" borderId="701" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="930" fillId="0" borderId="702" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="637" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="638" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="639" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="640" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="641" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="642" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="643" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="644" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="645" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="646" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="647" xfId="0"/>
+    <xf numFmtId="0" fontId="821" fillId="0" borderId="648" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="823" fillId="0" borderId="649" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="825" fillId="0" borderId="650" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="827" fillId="0" borderId="651" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="829" fillId="0" borderId="652" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="831" fillId="0" borderId="653" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="833" fillId="0" borderId="654" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="835" fillId="0" borderId="655" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="837" fillId="0" borderId="656" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="839" fillId="0" borderId="657" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="841" fillId="0" borderId="658" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="843" fillId="0" borderId="659" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="845" fillId="0" borderId="660" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="847" fillId="0" borderId="661" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="849" fillId="0" borderId="662" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="851" fillId="0" borderId="663" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="853" fillId="0" borderId="664" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="855" fillId="0" borderId="665" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="857" fillId="0" borderId="666" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="859" fillId="0" borderId="667" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="861" fillId="0" borderId="668" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="863" fillId="0" borderId="669" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="865" fillId="0" borderId="670" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="867" fillId="0" borderId="671" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="869" fillId="0" borderId="672" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="871" fillId="0" borderId="673" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="873" fillId="0" borderId="674" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="875" fillId="0" borderId="675" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="877" fillId="0" borderId="676" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="879" fillId="0" borderId="677" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="881" fillId="0" borderId="678" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="883" fillId="0" borderId="679" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="885" fillId="0" borderId="680" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="887" fillId="0" borderId="681" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="889" fillId="0" borderId="682" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="891" fillId="0" borderId="683" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="893" fillId="0" borderId="684" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="895" fillId="0" borderId="685" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="897" fillId="0" borderId="686" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="899" fillId="0" borderId="687" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="901" fillId="0" borderId="688" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="903" fillId="0" borderId="689" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="905" fillId="0" borderId="690" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="907" fillId="0" borderId="691" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="909" fillId="0" borderId="692" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="911" fillId="0" borderId="693" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="913" fillId="0" borderId="694" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="915" fillId="0" borderId="695" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="917" fillId="0" borderId="696" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="919" fillId="0" borderId="697" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="921" fillId="0" borderId="698" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="923" fillId="0" borderId="699" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="925" fillId="0" borderId="700" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="927" fillId="0" borderId="701" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="929" fillId="0" borderId="702" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -19288,283 +19613,283 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="978" fillId="0" borderId="749" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="980" fillId="0" borderId="750" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="982" fillId="0" borderId="751" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="984" fillId="0" borderId="752" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="986" fillId="0" borderId="753" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="988" fillId="0" borderId="754" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="990" fillId="0" borderId="755" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="992" fillId="0" borderId="756" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="994" fillId="0" borderId="757" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="996" fillId="0" borderId="758" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="998" fillId="0" borderId="759" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1000" fillId="0" borderId="760" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1002" fillId="0" borderId="761" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1004" fillId="0" borderId="762" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1006" fillId="0" borderId="763" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1008" fillId="0" borderId="764" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1009" fillId="0" borderId="765" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="977" fillId="0" borderId="749" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="978" fillId="0" borderId="750" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="979" fillId="0" borderId="751" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="980" fillId="0" borderId="752" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="981" fillId="0" borderId="753" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="982" fillId="0" borderId="754" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="983" fillId="0" borderId="755" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="984" fillId="0" borderId="756" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="985" fillId="0" borderId="757" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="986" fillId="0" borderId="758" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="987" fillId="0" borderId="759" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="989" fillId="0" borderId="760" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="991" fillId="0" borderId="761" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="993" fillId="0" borderId="762" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="995" fillId="0" borderId="763" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="997" fillId="0" borderId="764" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="999" fillId="0" borderId="765" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1001" fillId="0" borderId="766" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1003" fillId="0" borderId="767" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1005" fillId="0" borderId="768" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1007" fillId="0" borderId="769" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1009" fillId="0" borderId="770" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1011" fillId="0" borderId="771" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1013" fillId="0" borderId="772" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1015" fillId="0" borderId="773" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1017" fillId="0" borderId="774" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1019" fillId="0" borderId="775" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1020" fillId="0" borderId="776" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1010" fillId="0" borderId="766" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1021" fillId="0" borderId="777" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1011" fillId="0" borderId="767" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1022" fillId="0" borderId="778" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="768" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="769" xfId="0"/>
-    <xf numFmtId="0" fontId="1013" fillId="0" borderId="770" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1015" fillId="0" borderId="771" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1017" fillId="0" borderId="772" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1019" fillId="0" borderId="773" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1021" fillId="0" borderId="774" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1023" fillId="0" borderId="775" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1025" fillId="0" borderId="776" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1026" fillId="0" borderId="777" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="779" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="780" xfId="0"/>
+    <xf numFmtId="0" fontId="1024" fillId="0" borderId="781" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1026" fillId="0" borderId="782" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1028" fillId="0" borderId="783" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1030" fillId="0" borderId="784" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1032" fillId="0" borderId="785" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1034" fillId="0" borderId="786" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1036" fillId="0" borderId="787" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1037" fillId="0" borderId="788" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1027" fillId="0" borderId="778" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1038" fillId="0" borderId="789" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1028" fillId="0" borderId="779" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1039" fillId="0" borderId="790" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1029" fillId="0" borderId="780" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1040" fillId="0" borderId="791" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1030" fillId="0" borderId="781" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1041" fillId="0" borderId="792" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1031" fillId="0" borderId="782" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1042" fillId="0" borderId="793" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1032" fillId="0" borderId="783" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1043" fillId="0" borderId="794" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1033" fillId="0" borderId="784" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1034" fillId="0" borderId="785" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1035" fillId="0" borderId="786" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1036" fillId="0" borderId="787" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1037" fillId="0" borderId="788" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1038" fillId="0" borderId="789" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1039" fillId="0" borderId="790" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1044" fillId="0" borderId="795" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1045" fillId="0" borderId="796" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1046" fillId="0" borderId="797" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1047" fillId="0" borderId="798" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1048" fillId="0" borderId="799" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1049" fillId="0" borderId="800" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1050" fillId="0" borderId="801" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1040" fillId="0" borderId="791" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1051" fillId="0" borderId="802" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1041" fillId="0" borderId="792" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1052" fillId="0" borderId="803" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1042" fillId="0" borderId="793" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1053" fillId="0" borderId="804" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1043" fillId="0" borderId="794" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1054" fillId="0" borderId="805" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1044" fillId="0" borderId="795" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1055" fillId="0" borderId="806" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="796" xfId="0"/>
-    <xf numFmtId="0" fontId="1046" fillId="0" borderId="797" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1048" fillId="0" borderId="798" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1050" fillId="0" borderId="799" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1052" fillId="0" borderId="800" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1054" fillId="0" borderId="801" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1056" fillId="0" borderId="802" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1058" fillId="0" borderId="803" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1059" fillId="0" borderId="804" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="807" xfId="0"/>
+    <xf numFmtId="0" fontId="1057" fillId="0" borderId="808" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1059" fillId="0" borderId="809" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1061" fillId="0" borderId="810" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1063" fillId="0" borderId="811" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1065" fillId="0" borderId="812" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1067" fillId="0" borderId="813" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1069" fillId="0" borderId="814" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1070" fillId="0" borderId="815" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1060" fillId="0" borderId="805" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1071" fillId="0" borderId="816" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1061" fillId="0" borderId="806" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1072" fillId="0" borderId="817" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1062" fillId="0" borderId="807" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1073" fillId="0" borderId="818" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1063" fillId="0" borderId="808" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1074" fillId="0" borderId="819" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1064" fillId="0" borderId="809" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1075" fillId="0" borderId="820" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1065" fillId="0" borderId="810" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1066" fillId="0" borderId="811" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1067" fillId="0" borderId="812" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1068" fillId="0" borderId="813" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1069" fillId="0" borderId="814" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1070" fillId="0" borderId="815" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1071" fillId="0" borderId="816" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1072" fillId="0" borderId="817" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1073" fillId="0" borderId="818" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1074" fillId="0" borderId="819" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1075" fillId="0" borderId="820" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1076" fillId="0" borderId="821" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19572,43 +19897,43 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1077" fillId="0" borderId="822" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1078" fillId="0" borderId="823" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1079" fillId="0" borderId="824" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1080" fillId="0" borderId="825" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1081" fillId="0" borderId="826" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1082" fillId="0" borderId="827" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1083" fillId="0" borderId="828" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1084" fillId="0" borderId="829" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1085" fillId="0" borderId="830" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1086" fillId="0" borderId="831" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1083" fillId="0" borderId="828" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1084" fillId="0" borderId="829" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1085" fillId="0" borderId="830" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1086" fillId="0" borderId="831" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1087" fillId="0" borderId="832" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19620,7 +19945,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1089" fillId="0" borderId="834" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1090" fillId="0" borderId="835" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19636,7 +19961,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1093" fillId="0" borderId="838" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1094" fillId="0" borderId="839" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19648,47 +19973,47 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1096" fillId="0" borderId="841" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1097" fillId="0" borderId="842" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1098" fillId="0" borderId="843" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1099" fillId="0" borderId="844" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1100" fillId="0" borderId="845" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1101" fillId="0" borderId="846" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1102" fillId="0" borderId="847" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1103" fillId="0" borderId="848" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1104" fillId="0" borderId="849" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1105" fillId="0" borderId="850" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1106" fillId="0" borderId="851" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1107" fillId="0" borderId="852" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19720,47 +20045,47 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1114" fillId="0" borderId="859" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1115" fillId="0" borderId="860" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1116" fillId="0" borderId="861" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1117" fillId="0" borderId="862" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1118" fillId="0" borderId="863" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1119" fillId="0" borderId="864" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1120" fillId="0" borderId="865" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1121" fillId="0" borderId="866" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1122" fillId="0" borderId="867" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1123" fillId="0" borderId="868" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1124" fillId="0" borderId="869" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1125" fillId="0" borderId="870" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19772,7 +20097,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1127" fillId="0" borderId="872" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1128" fillId="0" borderId="873" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19788,7 +20113,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1131" fillId="0" borderId="876" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1132" fillId="0" borderId="877" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19800,51 +20125,51 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1134" fillId="0" borderId="879" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1135" fillId="0" borderId="880" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1136" fillId="0" borderId="881" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1137" fillId="0" borderId="882" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1138" fillId="0" borderId="883" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1135" fillId="0" borderId="880" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1136" fillId="0" borderId="881" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1137" fillId="0" borderId="882" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1138" fillId="0" borderId="883" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="0" fontId="1139" fillId="0" borderId="884" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1140" fillId="0" borderId="885" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1141" fillId="0" borderId="886" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1142" fillId="0" borderId="887" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1143" fillId="0" borderId="888" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1144" fillId="0" borderId="889" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1145" fillId="0" borderId="890" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1146" fillId="0" borderId="891" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19856,19 +20181,19 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1148" fillId="0" borderId="893" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1149" fillId="0" borderId="894" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1150" fillId="0" borderId="895" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1151" fillId="0" borderId="896" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1152" fillId="0" borderId="897" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -19876,523 +20201,523 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1153" fillId="0" borderId="898" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1154" fillId="0" borderId="899" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1155" fillId="0" borderId="900" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1156" fillId="0" borderId="901" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1157" fillId="0" borderId="902" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1158" fillId="0" borderId="903" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1159" fillId="0" borderId="904" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1154" fillId="0" borderId="899" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1160" fillId="0" borderId="905" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1155" fillId="0" borderId="900" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1161" fillId="0" borderId="906" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1156" fillId="0" borderId="901" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1162" fillId="0" borderId="907" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1157" fillId="0" borderId="902" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1163" fillId="0" borderId="908" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1158" fillId="0" borderId="903" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1164" fillId="0" borderId="909" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1165" fillId="0" borderId="910" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1166" fillId="0" borderId="911" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1167" fillId="0" borderId="912" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1168" fillId="0" borderId="913" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1169" fillId="0" borderId="914" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1159" fillId="0" borderId="904" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1160" fillId="0" borderId="905" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1161" fillId="0" borderId="906" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1162" fillId="0" borderId="907" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1163" fillId="0" borderId="908" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1170" fillId="0" borderId="915" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1171" fillId="0" borderId="916" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1172" fillId="0" borderId="917" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1173" fillId="0" borderId="918" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1174" fillId="0" borderId="919" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1164" fillId="0" borderId="909" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1165" fillId="0" borderId="910" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1166" fillId="0" borderId="911" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1167" fillId="0" borderId="912" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1169" fillId="0" borderId="913" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1171" fillId="0" borderId="914" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1173" fillId="0" borderId="915" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1175" fillId="0" borderId="916" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1177" fillId="0" borderId="917" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1179" fillId="0" borderId="918" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1181" fillId="0" borderId="919" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1183" fillId="0" borderId="920" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1185" fillId="0" borderId="921" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1187" fillId="0" borderId="922" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1189" fillId="0" borderId="923" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1191" fillId="0" borderId="924" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1193" fillId="0" borderId="925" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1195" fillId="0" borderId="926" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1196" fillId="0" borderId="927" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1175" fillId="0" borderId="920" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1176" fillId="0" borderId="921" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1177" fillId="0" borderId="922" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1178" fillId="0" borderId="923" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1179" fillId="0" borderId="924" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1180" fillId="0" borderId="925" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1181" fillId="0" borderId="926" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1182" fillId="0" borderId="927" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1183" fillId="0" borderId="928" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1185" fillId="0" borderId="929" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1187" fillId="0" borderId="930" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1189" fillId="0" borderId="931" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1191" fillId="0" borderId="932" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1193" fillId="0" borderId="933" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1195" fillId="0" borderId="934" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1197" fillId="0" borderId="935" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1199" fillId="0" borderId="936" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1201" fillId="0" borderId="937" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1203" fillId="0" borderId="938" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1205" fillId="0" borderId="939" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1207" fillId="0" borderId="940" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1209" fillId="0" borderId="941" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1211" fillId="0" borderId="942" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1212" fillId="0" borderId="943" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1197" fillId="0" borderId="928" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1213" fillId="0" borderId="944" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1198" fillId="0" borderId="929" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1214" fillId="0" borderId="945" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1199" fillId="0" borderId="930" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1215" fillId="0" borderId="946" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1200" fillId="0" borderId="931" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1216" fillId="0" borderId="947" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1201" fillId="0" borderId="932" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1217" fillId="0" borderId="948" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1202" fillId="0" borderId="933" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1218" fillId="0" borderId="949" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1203" fillId="0" borderId="934" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1219" fillId="0" borderId="950" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1204" fillId="0" borderId="935" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1220" fillId="0" borderId="951" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="936" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="937" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="938" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="939" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="940" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="941" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="942" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="943" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="944" xfId="0"/>
-    <xf numFmtId="0" fontId="1206" fillId="0" borderId="945" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1208" fillId="0" borderId="946" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1210" fillId="0" borderId="947" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1212" fillId="0" borderId="948" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1214" fillId="0" borderId="949" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1216" fillId="0" borderId="950" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1218" fillId="0" borderId="951" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1220" fillId="0" borderId="952" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1222" fillId="0" borderId="953" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1224" fillId="0" borderId="954" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1226" fillId="0" borderId="955" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1228" fillId="0" borderId="956" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1230" fillId="0" borderId="957" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1232" fillId="0" borderId="958" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1234" fillId="0" borderId="959" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1236" fillId="0" borderId="960" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1238" fillId="0" borderId="961" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1240" fillId="0" borderId="962" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1242" fillId="0" borderId="963" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1244" fillId="0" borderId="964" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1246" fillId="0" borderId="965" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1248" fillId="0" borderId="966" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1250" fillId="0" borderId="967" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1252" fillId="0" borderId="968" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1254" fillId="0" borderId="969" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1256" fillId="0" borderId="970" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1258" fillId="0" borderId="971" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1260" fillId="0" borderId="972" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1262" fillId="0" borderId="973" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1264" fillId="0" borderId="974" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1266" fillId="0" borderId="975" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1268" fillId="0" borderId="976" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1270" fillId="0" borderId="977" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1272" fillId="0" borderId="978" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1274" fillId="0" borderId="979" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1276" fillId="0" borderId="980" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1278" fillId="0" borderId="981" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1280" fillId="0" borderId="982" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1282" fillId="0" borderId="983" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1284" fillId="0" borderId="984" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1286" fillId="0" borderId="985" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1288" fillId="0" borderId="986" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1290" fillId="0" borderId="987" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1292" fillId="0" borderId="988" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1294" fillId="0" borderId="989" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1296" fillId="0" borderId="990" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1298" fillId="0" borderId="991" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1300" fillId="0" borderId="992" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1302" fillId="0" borderId="993" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1304" fillId="0" borderId="994" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1306" fillId="0" borderId="995" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1308" fillId="0" borderId="996" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1310" fillId="0" borderId="997" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1312" fillId="0" borderId="998" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1314" fillId="0" borderId="999" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1316" fillId="0" borderId="1000" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1318" fillId="0" borderId="1001" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1320" fillId="0" borderId="1002" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1322" fillId="0" borderId="1003" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1324" fillId="0" borderId="1004" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1326" fillId="0" borderId="1005" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1328" fillId="0" borderId="1006" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1330" fillId="0" borderId="1007" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1332" fillId="0" borderId="1008" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1334" fillId="0" borderId="1009" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1336" fillId="0" borderId="1010" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1338" fillId="0" borderId="1011" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1340" fillId="0" borderId="1012" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1342" fillId="0" borderId="1013" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1344" fillId="0" borderId="1014" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1346" fillId="0" borderId="1015" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1348" fillId="0" borderId="1016" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1350" fillId="0" borderId="1017" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1352" fillId="0" borderId="1018" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1354" fillId="0" borderId="1019" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1355" fillId="0" borderId="1020" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1356" fillId="0" borderId="1021" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1357" fillId="0" borderId="1022" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1358" fillId="0" borderId="1023" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1359" fillId="0" borderId="1024" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1360" fillId="0" borderId="1025" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1361" fillId="0" borderId="1026" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1362" fillId="0" borderId="1027" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1363" fillId="0" borderId="1028" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1364" fillId="0" borderId="1029" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1365" fillId="0" borderId="1030" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1366" fillId="0" borderId="1031" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1367" fillId="0" borderId="1032" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1368" fillId="0" borderId="1033" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1369" fillId="0" borderId="1034" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="952" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="953" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="954" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="955" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="956" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="957" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="958" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="959" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="960" xfId="0"/>
+    <xf numFmtId="0" fontId="1222" fillId="0" borderId="961" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1224" fillId="0" borderId="962" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1226" fillId="0" borderId="963" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1228" fillId="0" borderId="964" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1230" fillId="0" borderId="965" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1232" fillId="0" borderId="966" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1234" fillId="0" borderId="967" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1236" fillId="0" borderId="968" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1238" fillId="0" borderId="969" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1240" fillId="0" borderId="970" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1242" fillId="0" borderId="971" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1244" fillId="0" borderId="972" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1246" fillId="0" borderId="973" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1248" fillId="0" borderId="974" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1250" fillId="0" borderId="975" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1252" fillId="0" borderId="976" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1254" fillId="0" borderId="977" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1256" fillId="0" borderId="978" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1258" fillId="0" borderId="979" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1260" fillId="0" borderId="980" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1262" fillId="0" borderId="981" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1264" fillId="0" borderId="982" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1266" fillId="0" borderId="983" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1268" fillId="0" borderId="984" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1270" fillId="0" borderId="985" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1272" fillId="0" borderId="986" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1274" fillId="0" borderId="987" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1276" fillId="0" borderId="988" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1278" fillId="0" borderId="989" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1280" fillId="0" borderId="990" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1282" fillId="0" borderId="991" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1284" fillId="0" borderId="992" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1286" fillId="0" borderId="993" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1288" fillId="0" borderId="994" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1290" fillId="0" borderId="995" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1292" fillId="0" borderId="996" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1294" fillId="0" borderId="997" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1296" fillId="0" borderId="998" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1298" fillId="0" borderId="999" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1300" fillId="0" borderId="1000" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1302" fillId="0" borderId="1001" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1304" fillId="0" borderId="1002" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1306" fillId="0" borderId="1003" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1308" fillId="0" borderId="1004" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1310" fillId="0" borderId="1005" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1312" fillId="0" borderId="1006" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1314" fillId="0" borderId="1007" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1316" fillId="0" borderId="1008" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1318" fillId="0" borderId="1009" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1320" fillId="0" borderId="1010" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1322" fillId="0" borderId="1011" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1324" fillId="0" borderId="1012" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1326" fillId="0" borderId="1013" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1328" fillId="0" borderId="1014" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1330" fillId="0" borderId="1015" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1332" fillId="0" borderId="1016" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1334" fillId="0" borderId="1017" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1336" fillId="0" borderId="1018" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1338" fillId="0" borderId="1019" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1340" fillId="0" borderId="1020" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1342" fillId="0" borderId="1021" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1344" fillId="0" borderId="1022" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1346" fillId="0" borderId="1023" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1348" fillId="0" borderId="1024" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1350" fillId="0" borderId="1025" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1352" fillId="0" borderId="1026" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1354" fillId="0" borderId="1027" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1356" fillId="0" borderId="1028" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1358" fillId="0" borderId="1029" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1360" fillId="0" borderId="1030" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1362" fillId="0" borderId="1031" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1364" fillId="0" borderId="1032" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1366" fillId="0" borderId="1033" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1368" fillId="0" borderId="1034" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -20636,207 +20961,207 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1431" fillId="0" borderId="1095" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1433" fillId="0" borderId="1096" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1435" fillId="0" borderId="1097" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1437" fillId="0" borderId="1098" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1439" fillId="0" borderId="1099" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1441" fillId="0" borderId="1100" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1443" fillId="0" borderId="1101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1445" fillId="0" borderId="1102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1447" fillId="0" borderId="1103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1449" fillId="0" borderId="1104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1450" fillId="0" borderId="1105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1430" fillId="0" borderId="1095" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1431" fillId="0" borderId="1096" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1432" fillId="0" borderId="1097" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1433" fillId="0" borderId="1098" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1434" fillId="0" borderId="1099" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1435" fillId="0" borderId="1100" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1436" fillId="0" borderId="1101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1437" fillId="0" borderId="1102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1438" fillId="0" borderId="1103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1439" fillId="0" borderId="1104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1440" fillId="0" borderId="1105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1441" fillId="0" borderId="1106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1442" fillId="0" borderId="1107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1443" fillId="0" borderId="1108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1444" fillId="0" borderId="1109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1445" fillId="0" borderId="1110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1447" fillId="0" borderId="1111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1449" fillId="0" borderId="1112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1451" fillId="0" borderId="1113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1453" fillId="0" borderId="1114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1455" fillId="0" borderId="1115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1457" fillId="0" borderId="1116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1459" fillId="0" borderId="1117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1461" fillId="0" borderId="1118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1463" fillId="0" borderId="1119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1465" fillId="0" borderId="1120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1466" fillId="0" borderId="1121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1451" fillId="0" borderId="1106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1467" fillId="0" borderId="1122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1452" fillId="0" borderId="1107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1468" fillId="0" borderId="1123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1108" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1109" xfId="0"/>
-    <xf numFmtId="0" fontId="1454" fillId="0" borderId="1110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1456" fillId="0" borderId="1111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1458" fillId="0" borderId="1112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1460" fillId="0" borderId="1113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1461" fillId="0" borderId="1114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1124" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1125" xfId="0"/>
+    <xf numFmtId="0" fontId="1470" fillId="0" borderId="1126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1472" fillId="0" borderId="1127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1474" fillId="0" borderId="1128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1476" fillId="0" borderId="1129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1477" fillId="0" borderId="1130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1462" fillId="0" borderId="1115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1478" fillId="0" borderId="1131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1463" fillId="0" borderId="1116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1479" fillId="0" borderId="1132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1464" fillId="0" borderId="1117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1480" fillId="0" borderId="1133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1465" fillId="0" borderId="1118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1466" fillId="0" borderId="1119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1467" fillId="0" borderId="1120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1468" fillId="0" borderId="1121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1481" fillId="0" borderId="1134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1482" fillId="0" borderId="1135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1483" fillId="0" borderId="1136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1484" fillId="0" borderId="1137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1469" fillId="0" borderId="1122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1485" fillId="0" borderId="1138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1470" fillId="0" borderId="1123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1486" fillId="0" borderId="1139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1124" xfId="0"/>
-    <xf numFmtId="0" fontId="1472" fillId="0" borderId="1125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1474" fillId="0" borderId="1126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1476" fillId="0" borderId="1127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1478" fillId="0" borderId="1128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1479" fillId="0" borderId="1129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1140" xfId="0"/>
+    <xf numFmtId="0" fontId="1488" fillId="0" borderId="1141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1490" fillId="0" borderId="1142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1492" fillId="0" borderId="1143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1494" fillId="0" borderId="1144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1495" fillId="0" borderId="1145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1480" fillId="0" borderId="1130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1496" fillId="0" borderId="1146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1481" fillId="0" borderId="1131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1497" fillId="0" borderId="1147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1482" fillId="0" borderId="1132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1483" fillId="0" borderId="1133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1484" fillId="0" borderId="1134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1485" fillId="0" borderId="1135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1486" fillId="0" borderId="1136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1487" fillId="0" borderId="1137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1488" fillId="0" borderId="1138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1489" fillId="0" borderId="1139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1490" fillId="0" borderId="1140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1491" fillId="0" borderId="1141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1492" fillId="0" borderId="1142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1493" fillId="0" borderId="1143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1494" fillId="0" borderId="1144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1495" fillId="0" borderId="1145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1496" fillId="0" borderId="1146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1497" fillId="0" borderId="1147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1498" fillId="0" borderId="1148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -20844,59 +21169,59 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1499" fillId="0" borderId="1149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1500" fillId="0" borderId="1150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1501" fillId="0" borderId="1151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1502" fillId="0" borderId="1152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1503" fillId="0" borderId="1153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1504" fillId="0" borderId="1154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1505" fillId="0" borderId="1155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1506" fillId="0" borderId="1156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1507" fillId="0" borderId="1157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1508" fillId="0" borderId="1158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1509" fillId="0" borderId="1159" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1510" fillId="0" borderId="1160" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1511" fillId="0" borderId="1161" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1512" fillId="0" borderId="1162" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1513" fillId="0" borderId="1163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -21012,67 +21337,67 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1541" fillId="0" borderId="1191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1542" fillId="0" borderId="1192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1543" fillId="0" borderId="1193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1544" fillId="0" borderId="1194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1545" fillId="0" borderId="1195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1546" fillId="0" borderId="1196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1547" fillId="0" borderId="1197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1548" fillId="0" borderId="1198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1549" fillId="0" borderId="1199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1550" fillId="0" borderId="1200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1551" fillId="0" borderId="1201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1552" fillId="0" borderId="1202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1553" fillId="0" borderId="1203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1554" fillId="0" borderId="1204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1555" fillId="0" borderId="1205" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1556" fillId="0" borderId="1206" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1557" fillId="0" borderId="1207" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -21143,120 +21468,120 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1575" fillId="0" borderId="1224" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1576" fillId="0" borderId="1225" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1574" fillId="0" borderId="1224" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1575" fillId="0" borderId="1225" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1576" fillId="0" borderId="1226" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1577" fillId="0" borderId="1227" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1578" fillId="0" borderId="1228" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1579" fillId="0" borderId="1229" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1580" fillId="0" borderId="1230" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1581" fillId="0" borderId="1231" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1582" fillId="0" borderId="1232" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1583" fillId="0" borderId="1233" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1584" fillId="0" borderId="1234" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1585" fillId="0" borderId="1235" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1586" fillId="0" borderId="1236" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1587" fillId="0" borderId="1237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1588" fillId="0" borderId="1238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1589" fillId="0" borderId="1239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1591" fillId="0" borderId="1240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1592" fillId="0" borderId="1241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1577" fillId="0" borderId="1226" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1593" fillId="0" borderId="1242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1578" fillId="0" borderId="1227" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1594" fillId="0" borderId="1243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1579" fillId="0" borderId="1228" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1580" fillId="0" borderId="1229" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1581" fillId="0" borderId="1230" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1595" fillId="0" borderId="1244" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1596" fillId="0" borderId="1245" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1597" fillId="0" borderId="1246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1582" fillId="0" borderId="1231" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1598" fillId="0" borderId="1247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1583" fillId="0" borderId="1232" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1584" fillId="0" borderId="1233" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1585" fillId="0" borderId="1234" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1599" fillId="0" borderId="1248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1600" fillId="0" borderId="1249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1601" fillId="0" borderId="1250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1586" fillId="0" borderId="1235" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1602" fillId="0" borderId="1251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1587" fillId="0" borderId="1236" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1603" fillId="0" borderId="1252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1588" fillId="0" borderId="1237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1589" fillId="0" borderId="1238" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1590" fillId="0" borderId="1239" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1591" fillId="0" borderId="1240" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1592" fillId="0" borderId="1241" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1593" fillId="0" borderId="1242" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1594" fillId="0" borderId="1243" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1595" fillId="0" borderId="1244" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1596" fillId="0" borderId="1245" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1597" fillId="0" borderId="1246" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1598" fillId="0" borderId="1247" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1599" fillId="0" borderId="1248" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1600" fillId="0" borderId="1249" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1601" fillId="0" borderId="1250" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1602" fillId="0" borderId="1251" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1603" fillId="0" borderId="1252" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1604" fillId="0" borderId="1253" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -21264,47 +21589,47 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1605" fillId="0" borderId="1254" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1606" fillId="0" borderId="1255" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1607" fillId="0" borderId="1256" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1608" fillId="0" borderId="1257" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1606" fillId="0" borderId="1255" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1607" fillId="0" borderId="1256" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1608" fillId="0" borderId="1257" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="0" fontId="1609" fillId="0" borderId="1258" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1610" fillId="0" borderId="1259" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1611" fillId="0" borderId="1260" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1612" fillId="0" borderId="1261" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1613" fillId="0" borderId="1262" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1614" fillId="0" borderId="1263" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1615" fillId="0" borderId="1264" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1616" fillId="0" borderId="1265" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -21312,23 +21637,23 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1617" fillId="0" borderId="1266" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1618" fillId="0" borderId="1267" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1619" fillId="0" borderId="1268" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1620" fillId="0" borderId="1269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1618" fillId="0" borderId="1267" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1621" fillId="0" borderId="1270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1619" fillId="0" borderId="1268" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1620" fillId="0" borderId="1269" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1621" fillId="0" borderId="1270" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1622" fillId="0" borderId="1271" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -21364,119 +21689,235 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1630" fillId="0" borderId="1279" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1631" fillId="0" borderId="1280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1632" fillId="0" borderId="1281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1633" fillId="0" borderId="1282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1634" fillId="0" borderId="1283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1635" fillId="0" borderId="1284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1636" fillId="0" borderId="1285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1637" fillId="0" borderId="1286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1638" fillId="0" borderId="1287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1639" fillId="0" borderId="1288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1640" fillId="0" borderId="1289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1641" fillId="0" borderId="1290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1642" fillId="0" borderId="1291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1643" fillId="0" borderId="1292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1644" fillId="0" borderId="1293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1645" fillId="0" borderId="1294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1646" fillId="0" borderId="1295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1631" fillId="0" borderId="1280" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1632" fillId="0" borderId="1281" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1633" fillId="0" borderId="1282" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1634" fillId="0" borderId="1283" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1635" fillId="0" borderId="1284" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1636" fillId="0" borderId="1285" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1637" fillId="0" borderId="1286" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1638" fillId="0" borderId="1287" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1639" fillId="0" borderId="1288" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1640" fillId="0" borderId="1289" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1641" fillId="0" borderId="1290" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1642" fillId="0" borderId="1291" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1644" fillId="0" borderId="1292" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1646" fillId="0" borderId="1293" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1648" fillId="0" borderId="1294" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1650" fillId="0" borderId="1295" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1652" fillId="0" borderId="1296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1654" fillId="0" borderId="1297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1656" fillId="0" borderId="1298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1658" fillId="0" borderId="1299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1659" fillId="0" borderId="1300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1647" fillId="0" borderId="1296" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1648" fillId="0" borderId="1297" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1649" fillId="0" borderId="1298" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1650" fillId="0" borderId="1299" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1651" fillId="0" borderId="1300" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1652" fillId="0" borderId="1301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1653" fillId="0" borderId="1302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1654" fillId="0" borderId="1303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1655" fillId="0" borderId="1304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1656" fillId="0" borderId="1305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1657" fillId="0" borderId="1306" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1658" fillId="0" borderId="1307" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1659" fillId="0" borderId="1308" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1660" fillId="0" borderId="1309" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1661" fillId="0" borderId="1310" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1662" fillId="0" borderId="1311" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1663" fillId="0" borderId="1312" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1664" fillId="0" borderId="1313" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1665" fillId="0" borderId="1314" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1666" fillId="0" borderId="1315" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1667" fillId="0" borderId="1316" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1668" fillId="0" borderId="1317" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1669" fillId="0" borderId="1318" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1670" fillId="0" borderId="1319" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1671" fillId="0" borderId="1320" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1673" fillId="0" borderId="1321" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1675" fillId="0" borderId="1322" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1677" fillId="0" borderId="1323" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1679" fillId="0" borderId="1324" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1681" fillId="0" borderId="1325" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1683" fillId="0" borderId="1326" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1685" fillId="0" borderId="1327" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1687" fillId="0" borderId="1328" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1688" fillId="0" borderId="1329" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1660" fillId="0" borderId="1301" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1689" fillId="0" borderId="1330" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1661" fillId="0" borderId="1302" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1690" fillId="0" borderId="1331" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1662" fillId="0" borderId="1303" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1691" fillId="0" borderId="1332" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1663" fillId="0" borderId="1304" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1692" fillId="0" borderId="1333" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1664" fillId="0" borderId="1305" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="0" fontId="1693" fillId="0" borderId="1334" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1306" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1307" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1308" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1309" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1310" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1311" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1335" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1336" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1337" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1338" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1339" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1340" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21489,16 +21930,16 @@
   <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="627" customWidth="true"/>
-    <col min="2" max="2" width="24.7109375" style="628" customWidth="true"/>
-    <col min="3" max="3" width="17.7109375" style="629" customWidth="true"/>
-    <col min="4" max="4" width="15.7109375" style="630" customWidth="true"/>
-    <col min="5" max="5" width="15.7109375" style="631" customWidth="true"/>
-    <col min="6" max="6" width="9.7109375" style="632" customWidth="true"/>
-    <col min="7" max="7" width="8.7109375" style="633" customWidth="true"/>
-    <col min="8" max="8" width="9.7109375" style="634" customWidth="true"/>
-    <col min="9" max="9" width="8.7109375" style="635" customWidth="true"/>
-    <col min="10" max="10" width="9.7109375" style="636" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="638" customWidth="true"/>
+    <col min="2" max="2" width="24.7109375" style="639" customWidth="true"/>
+    <col min="3" max="3" width="17.7109375" style="640" customWidth="true"/>
+    <col min="4" max="4" width="15.7109375" style="641" customWidth="true"/>
+    <col min="5" max="5" width="15.7109375" style="642" customWidth="true"/>
+    <col min="6" max="6" width="9.7109375" style="643" customWidth="true"/>
+    <col min="7" max="7" width="8.7109375" style="644" customWidth="true"/>
+    <col min="8" max="8" width="9.7109375" style="645" customWidth="true"/>
+    <col min="9" max="9" width="8.7109375" style="646" customWidth="true"/>
+    <col min="10" max="10" width="9.7109375" style="647" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" s="284" customFormat="true" ht="30" customHeight="true">
@@ -21561,7 +22002,7 @@
       <c r="I2" s="533" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="534" t="s">
+      <c r="J2" s="597" t="s">
         <v>1</v>
       </c>
     </row>
@@ -21593,7 +22034,7 @@
       <c r="I3" s="542" t="s">
         <v>60</v>
       </c>
-      <c r="J3" s="543" t="s">
+      <c r="J3" s="598" t="s">
         <v>63</v>
       </c>
     </row>
@@ -21625,7 +22066,7 @@
       <c r="I4" s="443" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="444" t="s">
+      <c r="J4" s="599" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21657,7 +22098,7 @@
       <c r="I5" s="451" t="s">
         <v>61</v>
       </c>
-      <c r="J5" s="452" t="s">
+      <c r="J5" s="600" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21689,7 +22130,7 @@
       <c r="I6" s="459" t="s">
         <v>61</v>
       </c>
-      <c r="J6" s="460" t="s">
+      <c r="J6" s="601" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21721,7 +22162,7 @@
       <c r="I7" s="467" t="s">
         <v>61</v>
       </c>
-      <c r="J7" s="468" t="s">
+      <c r="J7" s="602" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21753,7 +22194,7 @@
       <c r="I8" s="475" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="476" t="s">
+      <c r="J8" s="603" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21785,7 +22226,7 @@
       <c r="I9" s="483" t="s">
         <v>61</v>
       </c>
-      <c r="J9" s="484" t="s">
+      <c r="J9" s="604" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21817,7 +22258,7 @@
       <c r="I10" s="491" t="s">
         <v>61</v>
       </c>
-      <c r="J10" s="492" t="s">
+      <c r="J10" s="605" t="s">
         <v>64</v>
       </c>
     </row>
@@ -21849,7 +22290,7 @@
       <c r="I11" s="499" t="s">
         <v>62</v>
       </c>
-      <c r="J11" s="500" t="s">
+      <c r="J11" s="606" t="s">
         <v>65</v>
       </c>
     </row>
@@ -21881,39 +22322,39 @@
       <c r="I12" s="551" t="s">
         <v>62</v>
       </c>
-      <c r="J12" s="552" t="s">
+      <c r="J12" s="607" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="13" s="626" customFormat="true" ht="38" customHeight="true">
+    <row r="13" s="637" customFormat="true" ht="38" customHeight="true">
       <c r="A13" s="251" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="625" t="s">
+      <c r="B13" s="636" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="616" t="s">
+      <c r="C13" s="627" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="617" t="s">
+      <c r="D13" s="628" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="618" t="s">
+      <c r="E13" s="629" t="s">
         <v>1</v>
       </c>
-      <c r="F13" s="619" t="s">
+      <c r="F13" s="630" t="s">
         <v>1</v>
       </c>
-      <c r="G13" s="620" t="s">
+      <c r="G13" s="631" t="s">
         <v>1</v>
       </c>
-      <c r="H13" s="621" t="s">
+      <c r="H13" s="632" t="s">
         <v>1</v>
       </c>
-      <c r="I13" s="622" t="s">
+      <c r="I13" s="633" t="s">
         <v>1</v>
       </c>
-      <c r="J13" s="623" t="s">
+      <c r="J13" s="634" t="s">
         <v>1</v>
       </c>
     </row>
@@ -21933,195 +22374,195 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="937" customWidth="true"/>
-    <col min="2" max="2" width="36.7109375" style="938" customWidth="true"/>
-    <col min="3" max="3" width="10.7109375" style="939" customWidth="true"/>
-    <col min="4" max="4" width="16.7109375" style="940" customWidth="true"/>
-    <col min="5" max="5" width="9.7109375" style="941" customWidth="true"/>
-    <col min="6" max="6" width="10.7109375" style="942" customWidth="true"/>
-    <col min="7" max="7" width="16.7109375" style="943" customWidth="true"/>
-    <col min="8" max="8" width="9.7109375" style="944" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="953" customWidth="true"/>
+    <col min="2" max="2" width="36.7109375" style="954" customWidth="true"/>
+    <col min="3" max="3" width="10.7109375" style="955" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" style="956" customWidth="true"/>
+    <col min="5" max="5" width="9.7109375" style="957" customWidth="true"/>
+    <col min="6" max="6" width="10.7109375" style="958" customWidth="true"/>
+    <col min="7" max="7" width="16.7109375" style="959" customWidth="true"/>
+    <col min="8" max="8" width="9.7109375" style="960" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="768" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="767" t="s">
+    <row r="1" s="779" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="778" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="757" t="s">
+      <c r="B1" s="768" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="757" t="s">
+      <c r="C1" s="768" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="757" t="s">
+      <c r="D1" s="768" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="757" t="s">
+      <c r="E1" s="768" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="757" t="s">
+      <c r="F1" s="768" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="757" t="s">
+      <c r="G1" s="768" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="757" t="s">
+      <c r="H1" s="768" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" s="796" customFormat="true" ht="24" customHeight="true">
-      <c r="A2" s="701" t="s">
+    <row r="2" s="807" customFormat="true" ht="24" customHeight="true">
+      <c r="A2" s="712" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="898" t="s">
+      <c r="B2" s="909" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="873" t="s">
+      <c r="C2" s="884" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="874" t="s">
+      <c r="D2" s="885" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="903" t="s">
+      <c r="E2" s="914" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="876" t="s">
+      <c r="F2" s="887" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="877" t="s">
+      <c r="G2" s="888" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="908" t="s">
+      <c r="H2" s="924" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="709" t="s">
+      <c r="A3" s="720" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="899" t="s">
+      <c r="B3" s="910" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="880" t="s">
+      <c r="C3" s="891" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="881" t="s">
+      <c r="D3" s="892" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="904" t="s">
+      <c r="E3" s="915" t="s">
         <v>78</v>
       </c>
-      <c r="F3" s="883" t="s">
+      <c r="F3" s="894" t="s">
         <v>72</v>
       </c>
-      <c r="G3" s="884" t="s">
+      <c r="G3" s="895" t="s">
         <v>75</v>
       </c>
-      <c r="H3" s="909" t="s">
+      <c r="H3" s="925" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="717" t="s">
+      <c r="A4" s="728" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="900" t="s">
+      <c r="B4" s="911" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="841" t="s">
+      <c r="C4" s="852" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="842" t="s">
+      <c r="D4" s="853" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="905" t="s">
+      <c r="E4" s="916" t="s">
         <v>79</v>
       </c>
-      <c r="F4" s="844" t="s">
+      <c r="F4" s="855" t="s">
         <v>82</v>
       </c>
-      <c r="G4" s="845" t="s">
+      <c r="G4" s="856" t="s">
         <v>84</v>
       </c>
-      <c r="H4" s="910" t="s">
+      <c r="H4" s="926" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="725" t="s">
+      <c r="A5" s="736" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="901" t="s">
+      <c r="B5" s="912" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="847" t="s">
+      <c r="C5" s="858" t="s">
         <v>74</v>
       </c>
-      <c r="D5" s="848" t="s">
+      <c r="D5" s="859" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="906" t="s">
+      <c r="E5" s="917" t="s">
         <v>80</v>
       </c>
-      <c r="F5" s="850" t="s">
+      <c r="F5" s="861" t="s">
         <v>83</v>
       </c>
-      <c r="G5" s="851" t="s">
+      <c r="G5" s="862" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="911" t="s">
+      <c r="H5" s="927" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="733" t="s">
+      <c r="A6" s="744" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="902" t="s">
+      <c r="B6" s="913" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="887" t="s">
+      <c r="C6" s="898" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="888" t="s">
+      <c r="D6" s="899" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="907" t="s">
+      <c r="E6" s="918" t="s">
         <v>79</v>
       </c>
-      <c r="F6" s="890" t="s">
+      <c r="F6" s="901" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="891" t="s">
+      <c r="G6" s="902" t="s">
         <v>1</v>
       </c>
-      <c r="H6" s="912" t="s">
+      <c r="H6" s="928" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="7" s="936" customFormat="true" ht="38" customHeight="true">
-      <c r="A7" s="741" t="s">
+    <row r="7" s="952" customFormat="true" ht="38" customHeight="true">
+      <c r="A7" s="752" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="935" t="s">
+      <c r="B7" s="951" t="s">
         <v>70</v>
       </c>
-      <c r="C7" s="928" t="s">
+      <c r="C7" s="944" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="929" t="s">
+      <c r="D7" s="945" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="930" t="s">
+      <c r="E7" s="946" t="s">
         <v>1</v>
       </c>
-      <c r="F7" s="931" t="s">
+      <c r="F7" s="947" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="932" t="s">
+      <c r="G7" s="948" t="s">
         <v>1</v>
       </c>
-      <c r="H7" s="933" t="s">
+      <c r="H7" s="949" t="s">
         <v>1</v>
       </c>
     </row>
@@ -22140,265 +22581,265 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" style="1307" customWidth="true"/>
-    <col min="2" max="2" width="30.7109375" style="1308" customWidth="true"/>
-    <col min="3" max="3" width="18.7109375" style="1309" customWidth="true"/>
-    <col min="4" max="4" width="8.7109375" style="1310" customWidth="true"/>
-    <col min="5" max="5" width="18.7109375" style="1311" customWidth="true"/>
+    <col min="1" max="1" width="1.7109375" style="1336" customWidth="true"/>
+    <col min="2" max="2" width="30.7109375" style="1337" customWidth="true"/>
+    <col min="3" max="3" width="18.7109375" style="1338" customWidth="true"/>
+    <col min="4" max="4" width="8.7109375" style="1339" customWidth="true"/>
+    <col min="5" max="5" width="18.7109375" style="1340" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="1108" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="1107" t="s">
+    <row r="1" s="1124" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="1123" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="1100" t="s">
+      <c r="B1" s="1116" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1100" t="s">
+      <c r="C1" s="1116" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1100" t="s">
+      <c r="D1" s="1116" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1100" t="s">
+      <c r="E1" s="1116" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" s="1124" customFormat="true" ht="24" customHeight="true">
-      <c r="A2" s="1025" t="s">
+    <row r="2" s="1140" customFormat="true" ht="24" customHeight="true">
+      <c r="A2" s="1041" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1266" t="s">
+      <c r="B2" s="1282" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1242" t="s">
+      <c r="C2" s="1258" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="1243" t="s">
+      <c r="D2" s="1259" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="1279" t="s">
+      <c r="E2" s="1308" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1030" t="s">
+      <c r="A3" s="1046" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1267" t="s">
+      <c r="B3" s="1283" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="1246" t="s">
+      <c r="C3" s="1262" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="1247" t="s">
+      <c r="D3" s="1263" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="1280" t="s">
+      <c r="E3" s="1309" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1035" t="s">
+      <c r="A4" s="1051" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="1268" t="s">
+      <c r="B4" s="1284" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="1191" t="s">
+      <c r="C4" s="1207" t="s">
         <v>102</v>
       </c>
-      <c r="D4" s="1192" t="s">
+      <c r="D4" s="1208" t="s">
         <v>112</v>
       </c>
-      <c r="E4" s="1281" t="s">
+      <c r="E4" s="1310" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1040" t="s">
+      <c r="A5" s="1056" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="1269" t="s">
+      <c r="B5" s="1285" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="1194" t="s">
+      <c r="C5" s="1210" t="s">
         <v>103</v>
       </c>
-      <c r="D5" s="1195" t="s">
+      <c r="D5" s="1211" t="s">
         <v>113</v>
       </c>
-      <c r="E5" s="1282" t="s">
+      <c r="E5" s="1311" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1045" t="s">
+      <c r="A6" s="1061" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="1270" t="s">
+      <c r="B6" s="1286" t="s">
         <v>91</v>
       </c>
-      <c r="C6" s="1197" t="s">
+      <c r="C6" s="1213" t="s">
         <v>104</v>
       </c>
-      <c r="D6" s="1198" t="s">
+      <c r="D6" s="1214" t="s">
         <v>114</v>
       </c>
-      <c r="E6" s="1283" t="s">
+      <c r="E6" s="1312" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1050" t="s">
+      <c r="A7" s="1066" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="1271" t="s">
+      <c r="B7" s="1287" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="1231" t="s">
+      <c r="C7" s="1247" t="s">
         <v>105</v>
       </c>
-      <c r="D7" s="1232" t="s">
+      <c r="D7" s="1248" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="1284" t="s">
+      <c r="E7" s="1313" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1055" t="s">
+      <c r="A8" s="1071" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="1272" t="s">
+      <c r="B8" s="1288" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="1203" t="s">
+      <c r="C8" s="1219" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="1204" t="s">
+      <c r="D8" s="1220" t="s">
         <v>1</v>
       </c>
-      <c r="E8" s="1285" t="s">
+      <c r="E8" s="1314" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1060" t="s">
+      <c r="A9" s="1076" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="1273" t="s">
+      <c r="B9" s="1289" t="s">
         <v>93</v>
       </c>
-      <c r="C9" s="1206" t="s">
+      <c r="C9" s="1222" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="1207" t="s">
+      <c r="D9" s="1223" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="1286" t="s">
+      <c r="E9" s="1315" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1065" t="s">
+      <c r="A10" s="1081" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="1274" t="s">
+      <c r="B10" s="1290" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="1209" t="s">
+      <c r="C10" s="1225" t="s">
         <v>108</v>
       </c>
-      <c r="D10" s="1210" t="s">
+      <c r="D10" s="1226" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="1287" t="s">
+      <c r="E10" s="1316" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1070" t="s">
+      <c r="A11" s="1086" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="1275" t="s">
+      <c r="B11" s="1291" t="s">
         <v>95</v>
       </c>
-      <c r="C11" s="1212" t="s">
+      <c r="C11" s="1228" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="1213" t="s">
+      <c r="D11" s="1229" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="1288" t="s">
+      <c r="E11" s="1317" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1075" t="s">
+      <c r="A12" s="1091" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="1276" t="s">
+      <c r="B12" s="1292" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="1215" t="s">
+      <c r="C12" s="1231" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="1216" t="s">
+      <c r="D12" s="1232" t="s">
         <v>1</v>
       </c>
-      <c r="E12" s="1289" t="s">
+      <c r="E12" s="1318" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1080" t="s">
+      <c r="A13" s="1096" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="1277" t="s">
+      <c r="B13" s="1293" t="s">
         <v>97</v>
       </c>
-      <c r="C13" s="1218" t="s">
+      <c r="C13" s="1234" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="1219" t="s">
+      <c r="D13" s="1235" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="1290" t="s">
+      <c r="E13" s="1319" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1085" t="s">
+      <c r="A14" s="1101" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="1278" t="s">
+      <c r="B14" s="1294" t="s">
         <v>98</v>
       </c>
-      <c r="C14" s="1250" t="s">
+      <c r="C14" s="1266" t="s">
         <v>103</v>
       </c>
-      <c r="D14" s="1251" t="s">
+      <c r="D14" s="1267" t="s">
         <v>1</v>
       </c>
-      <c r="E14" s="1291" t="s">
+      <c r="E14" s="1320" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="15" s="1306" customFormat="true" ht="38" customHeight="true">
-      <c r="A15" s="1090" t="s">
+    <row r="15" s="1335" customFormat="true" ht="38" customHeight="true">
+      <c r="A15" s="1106" t="s">
         <v>1</v>
       </c>
-      <c r="B15" s="1305" t="s">
+      <c r="B15" s="1334" t="s">
         <v>99</v>
       </c>
-      <c r="C15" s="1301" t="s">
+      <c r="C15" s="1330" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="1302" t="s">
+      <c r="D15" s="1331" t="s">
         <v>1</v>
       </c>
-      <c r="E15" s="1303" t="s">
+      <c r="E15" s="1332" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finegray/iivw: add Fine-Gray tie-handling QA suite and refresh demo o...
</commit_message>
<xml_diff>
--- a/iivw/demo/iivw_reporting_exports.xlsx
+++ b/iivw/demo/iivw_reporting_exports.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="261" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="261" uniqueCount="122">
   <si>
     <t>IIVW balance diagnostic</t>
   </si>
@@ -53,7 +53,7 @@
     <t>relapse_lag1</t>
   </si>
   <si>
-    <t>Modeled identifies visit-intensity model covariates; |SMD| is the absolute weighted-minus-unweighted standardized difference.</t>
+    <t>Modeled identifies visit-intensity model covariates. Shift is the weighted-minus-unweighted mean in unweighted SD units: it measures how far the weights moved the composition of the observed visits, and is descriptive only. The balance verdict comes from the residual coefficients of the IIW-weighted visit-model refit.</t>
   </si>
   <si>
     <t>Means</t>
@@ -92,31 +92,31 @@
     <t>Weighted mean</t>
   </si>
   <si>
-    <t>0.6391</t>
+    <t>0.6386</t>
   </si>
   <si>
-    <t>39.8660</t>
+    <t>39.6832</t>
   </si>
   <si>
-    <t>0.6496</t>
+    <t>0.6402</t>
   </si>
   <si>
-    <t>2.2839</t>
+    <t>2.1938</t>
   </si>
   <si>
-    <t>48.9014</t>
+    <t>49.0273</t>
   </si>
   <si>
-    <t>6.7674</t>
+    <t>6.7053</t>
   </si>
   <si>
-    <t>0.3998</t>
+    <t>0.3865</t>
   </si>
   <si>
-    <t>52.8574</t>
+    <t>53.0730</t>
   </si>
   <si>
-    <t>0.2051</t>
+    <t>0.1919</t>
   </si>
   <si>
     <t>Unweighted SD</t>
@@ -149,43 +149,55 @@
     <t>0.3972</t>
   </si>
   <si>
-    <t>Balance</t>
+    <t>Composition shift</t>
   </si>
   <si>
-    <t>SMD</t>
+    <t>Shift</t>
   </si>
   <si>
-    <t>0.0030</t>
+    <t>0.0021</t>
   </si>
   <si>
-    <t>0.0359</t>
+    <t>0.0095</t>
   </si>
   <si>
-    <t>0.0082</t>
+    <t>-0.0116</t>
   </si>
   <si>
-    <t>0.0740</t>
+    <t>-0.0273</t>
   </si>
   <si>
-    <t>-0.0246</t>
+    <t>-0.0035</t>
   </si>
   <si>
-    <t>0.0140</t>
+    <t>-0.0044</t>
   </si>
   <si>
-    <t>0.0361</t>
+    <t>0.0087</t>
   </si>
   <si>
-    <t>0.0209</t>
+    <t>0.0538</t>
   </si>
   <si>
-    <t>0.0226</t>
+    <t>-0.0107</t>
   </si>
   <si>
-    <t>|SMD|</t>
+    <t>|Shift|</t>
   </si>
   <si>
-    <t>0.0246</t>
+    <t>0.0116</t>
+  </si>
+  <si>
+    <t>0.0273</t>
+  </si>
+  <si>
+    <t>0.0035</t>
+  </si>
+  <si>
+    <t>0.0044</t>
+  </si>
+  <si>
+    <t>0.0107</t>
   </si>
   <si>
     <t>Modeled</t>
@@ -236,19 +248,19 @@
     <t>HR</t>
   </si>
   <si>
-    <t>0.956</t>
+    <t>0.951</t>
   </si>
   <si>
-    <t>1.043</t>
+    <t>1.103</t>
   </si>
   <si>
     <t>95% CI</t>
   </si>
   <si>
-    <t>(0.937, 0.975)</t>
+    <t>(0.923, 0.979)</t>
   </si>
   <si>
-    <t>(0.923, 1.179)</t>
+    <t>(0.957, 1.273)</t>
   </si>
   <si>
     <t>p-value</t>
@@ -257,25 +269,28 @@
     <t>&lt;0.001</t>
   </si>
   <si>
-    <t>0.501</t>
+    <t>0.177</t>
+  </si>
+  <si>
+    <t>0.001</t>
   </si>
   <si>
     <t>NTZ-like</t>
   </si>
   <si>
-    <t>0.947</t>
+    <t>0.943</t>
   </si>
   <si>
-    <t>0.957</t>
+    <t>0.987</t>
   </si>
   <si>
-    <t>(0.936, 0.958)</t>
+    <t>(0.929, 0.958)</t>
   </si>
   <si>
-    <t>(0.897, 1.020)</t>
+    <t>(0.905, 1.075)</t>
   </si>
   <si>
-    <t>0.175</t>
+    <t>0.757</t>
   </si>
   <si>
     <t>IIVW diagnostic decomposition</t>
@@ -326,28 +341,25 @@
     <t>0.7262</t>
   </si>
   <si>
-    <t>0.6566</t>
+    <t>0.7264</t>
   </si>
   <si>
-    <t>-0.4833</t>
+    <t>-0.3872</t>
   </si>
   <si>
     <t>Diagnostic values</t>
   </si>
   <si>
-    <t>0.0696</t>
+    <t>-0.0002</t>
   </si>
   <si>
-    <t>1.1398</t>
+    <t>1.1136</t>
   </si>
   <si>
-    <t>1.2094</t>
+    <t>1.1134</t>
   </si>
   <si>
-    <t>0.0575</t>
-  </si>
-  <si>
-    <t>0.9425</t>
+    <t>1.0002</t>
   </si>
   <si>
     <t>SE</t>
@@ -356,19 +368,19 @@
     <t>0.0860</t>
   </si>
   <si>
-    <t>0.0826</t>
+    <t>0.0838</t>
   </si>
   <si>
-    <t>0.2235</t>
+    <t>0.2231</t>
   </si>
   <si>
     <t>0.5577 to 0.8947</t>
   </si>
   <si>
-    <t>0.4947 to 0.8185</t>
+    <t>0.5622 to 0.8906</t>
   </si>
   <si>
-    <t>-0.9213 to -0.0453</t>
+    <t>-0.8244 to 0.0500</t>
   </si>
 </sst>
 </file>
@@ -21935,8 +21947,8 @@
     <col min="3" max="3" width="17.7109375" style="640" customWidth="true"/>
     <col min="4" max="4" width="15.7109375" style="641" customWidth="true"/>
     <col min="5" max="5" width="15.7109375" style="642" customWidth="true"/>
-    <col min="6" max="6" width="9.7109375" style="643" customWidth="true"/>
-    <col min="7" max="7" width="8.7109375" style="644" customWidth="true"/>
+    <col min="6" max="6" width="18.7109375" style="643" customWidth="true"/>
+    <col min="7" max="7" width="9.7109375" style="644" customWidth="true"/>
     <col min="8" max="8" width="9.7109375" style="645" customWidth="true"/>
     <col min="9" max="9" width="8.7109375" style="646" customWidth="true"/>
     <col min="10" max="10" width="9.7109375" style="647" customWidth="true"/>
@@ -22000,7 +22012,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="533" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J2" s="597" t="s">
         <v>1</v>
@@ -22029,13 +22041,13 @@
         <v>55</v>
       </c>
       <c r="H3" s="587" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I3" s="542" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="J3" s="598" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4">
@@ -22061,13 +22073,13 @@
         <v>46</v>
       </c>
       <c r="H4" s="588" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I4" s="443" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J4" s="599" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
@@ -22093,13 +22105,13 @@
         <v>47</v>
       </c>
       <c r="H5" s="589" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I5" s="451" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J5" s="600" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6">
@@ -22122,16 +22134,16 @@
         <v>48</v>
       </c>
       <c r="G6" s="457" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="H6" s="590" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I6" s="459" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J6" s="601" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7">
@@ -22154,16 +22166,16 @@
         <v>49</v>
       </c>
       <c r="G7" s="465" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="H7" s="591" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I7" s="467" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J7" s="602" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8">
@@ -22186,16 +22198,16 @@
         <v>50</v>
       </c>
       <c r="G8" s="473" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H8" s="592" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I8" s="475" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J8" s="603" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9">
@@ -22218,16 +22230,16 @@
         <v>51</v>
       </c>
       <c r="G9" s="481" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H9" s="593" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I9" s="483" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J9" s="604" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10">
@@ -22253,13 +22265,13 @@
         <v>52</v>
       </c>
       <c r="H10" s="594" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I10" s="491" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="J10" s="605" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11">
@@ -22285,13 +22297,13 @@
         <v>53</v>
       </c>
       <c r="H11" s="595" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I11" s="499" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J11" s="606" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -22314,16 +22326,16 @@
         <v>54</v>
       </c>
       <c r="G12" s="549" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="H12" s="596" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I12" s="551" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J12" s="607" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" s="637" customFormat="true" ht="38" customHeight="true">
@@ -22386,7 +22398,7 @@
   <sheetData>
     <row r="1" s="779" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="778" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B1" s="768" t="s">
         <v>1</v>
@@ -22418,7 +22430,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="884" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D2" s="885" t="s">
         <v>1</v>
@@ -22427,7 +22439,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="887" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="G2" s="888" t="s">
         <v>1</v>
@@ -22444,22 +22456,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="891" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D3" s="892" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E3" s="915" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F3" s="894" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G3" s="895" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H3" s="925" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
@@ -22467,25 +22479,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="911" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C4" s="852" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D4" s="853" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E4" s="916" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F4" s="855" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G4" s="856" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H4" s="926" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5">
@@ -22493,25 +22505,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="912" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C5" s="858" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D5" s="859" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E5" s="917" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F5" s="861" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="G5" s="862" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H5" s="927" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6">
@@ -22519,7 +22531,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="913" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C6" s="898" t="s">
         <v>1</v>
@@ -22528,7 +22540,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="918" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F6" s="901" t="s">
         <v>1</v>
@@ -22537,7 +22549,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="928" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" s="952" customFormat="true" ht="38" customHeight="true">
@@ -22545,7 +22557,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="951" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C7" s="944" t="s">
         <v>1</v>
@@ -22590,7 +22602,7 @@
   <sheetData>
     <row r="1" s="1124" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="1123" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1116" t="s">
         <v>1</v>
@@ -22613,7 +22625,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1258" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D2" s="1259" t="s">
         <v>1</v>
@@ -22627,16 +22639,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="1283" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C3" s="1262" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D3" s="1263" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E3" s="1309" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4">
@@ -22644,16 +22656,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="1284" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C4" s="1207" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D4" s="1208" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E4" s="1310" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5">
@@ -22661,16 +22673,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="1285" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C5" s="1210" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D5" s="1211" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E5" s="1311" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -22678,16 +22690,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="1286" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C6" s="1213" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D6" s="1214" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E6" s="1312" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7">
@@ -22698,7 +22710,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="1247" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D7" s="1248" t="s">
         <v>1</v>
@@ -22712,10 +22724,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="1288" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C8" s="1219" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D8" s="1220" t="s">
         <v>1</v>
@@ -22729,10 +22741,10 @@
         <v>1</v>
       </c>
       <c r="B9" s="1289" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C9" s="1222" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D9" s="1223" t="s">
         <v>1</v>
@@ -22746,10 +22758,10 @@
         <v>1</v>
       </c>
       <c r="B10" s="1290" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C10" s="1225" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D10" s="1226" t="s">
         <v>1</v>
@@ -22763,10 +22775,10 @@
         <v>1</v>
       </c>
       <c r="B11" s="1291" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C11" s="1228" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D11" s="1229" t="s">
         <v>1</v>
@@ -22780,10 +22792,10 @@
         <v>1</v>
       </c>
       <c r="B12" s="1292" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C12" s="1231" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D12" s="1232" t="s">
         <v>1</v>
@@ -22797,10 +22809,10 @@
         <v>1</v>
       </c>
       <c r="B13" s="1293" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C13" s="1234" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D13" s="1235" t="s">
         <v>1</v>
@@ -22814,10 +22826,10 @@
         <v>1</v>
       </c>
       <c r="B14" s="1294" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C14" s="1266" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D14" s="1267" t="s">
         <v>1</v>
@@ -22831,7 +22843,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="1334" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C15" s="1330" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
iivw: broaden coverage, add FIPTIW interval QA and demo updates
</commit_message>
<xml_diff>
--- a/iivw/demo/iivw_reporting_exports.xlsx
+++ b/iivw/demo/iivw_reporting_exports.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="261" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="261" uniqueCount="124">
   <si>
     <t>IIVW balance diagnostic</t>
   </si>
@@ -53,7 +53,7 @@
     <t>relapse_lag1</t>
   </si>
   <si>
-    <t>Modeled identifies visit-intensity model covariates. Shift is the weighted-minus-unweighted mean in unweighted SD units: it measures how far the weights moved the composition of the observed visits, and is descriptive only. The balance verdict comes from the residual coefficients of the IIW-weighted visit-model refit.</t>
+    <t>Modeled identifies visit-intensity model covariates. Shift is the weighted-minus-unweighted mean in unweighted SD units: it measures how far the weights moved the composition of the observed visits, and is descriptive only. The balance verdict comes from Target SMD -- the IIW-weighted mean over observed visits against the person-time mean implied by the replayed visit model -- compared with balcut(). The visit model is replayed on all stored rows; if/in restricts this report only. Target status: identified.</t>
   </si>
   <si>
     <t>Means</t>
@@ -92,25 +92,25 @@
     <t>Weighted mean</t>
   </si>
   <si>
-    <t>0.6386</t>
+    <t>0.6367</t>
   </si>
   <si>
-    <t>39.6832</t>
+    <t>39.6869</t>
   </si>
   <si>
     <t>0.6402</t>
   </si>
   <si>
-    <t>2.1938</t>
+    <t>2.1933</t>
   </si>
   <si>
-    <t>49.0273</t>
+    <t>49.0275</t>
   </si>
   <si>
-    <t>6.7053</t>
+    <t>6.7065</t>
   </si>
   <si>
-    <t>0.3865</t>
+    <t>0.3867</t>
   </si>
   <si>
     <t>53.0730</t>
@@ -155,25 +155,25 @@
     <t>Shift</t>
   </si>
   <si>
-    <t>0.0021</t>
+    <t>-0.0019</t>
   </si>
   <si>
-    <t>0.0095</t>
+    <t>0.0100</t>
   </si>
   <si>
     <t>-0.0116</t>
   </si>
   <si>
-    <t>-0.0273</t>
+    <t>-0.0279</t>
   </si>
   <si>
     <t>-0.0035</t>
   </si>
   <si>
-    <t>-0.0044</t>
+    <t>-0.0041</t>
   </si>
   <si>
-    <t>0.0087</t>
+    <t>0.0091</t>
   </si>
   <si>
     <t>0.0538</t>
@@ -185,16 +185,19 @@
     <t>|Shift|</t>
   </si>
   <si>
+    <t>0.0019</t>
+  </si>
+  <si>
     <t>0.0116</t>
   </si>
   <si>
-    <t>0.0273</t>
+    <t>0.0279</t>
   </si>
   <si>
     <t>0.0035</t>
   </si>
   <si>
-    <t>0.0044</t>
+    <t>0.0041</t>
   </si>
   <si>
     <t>0.0107</t>
@@ -323,10 +326,10 @@
     <t>Artifact share</t>
   </si>
   <si>
-    <t>Lower bound</t>
+    <t>Range min</t>
   </si>
   <si>
-    <t>Upper bound</t>
+    <t>Range max</t>
   </si>
   <si>
     <t>Estimate rows report b, SE, and confidence limits; diagnostic and bias rows report a single value below the Diagnostic values divider.</t>
@@ -341,25 +344,28 @@
     <t>0.7262</t>
   </si>
   <si>
-    <t>0.7264</t>
+    <t>0.7337</t>
   </si>
   <si>
-    <t>-0.3872</t>
+    <t>-0.3802</t>
   </si>
   <si>
     <t>Diagnostic values</t>
   </si>
   <si>
-    <t>-0.0002</t>
+    <t>-0.0075</t>
   </si>
   <si>
-    <t>1.1136</t>
+    <t>1.1138</t>
   </si>
   <si>
-    <t>1.1134</t>
+    <t>1.1064</t>
   </si>
   <si>
-    <t>1.0002</t>
+    <t>-0.0068</t>
+  </si>
+  <si>
+    <t>1.0068</t>
   </si>
   <si>
     <t>SE</t>
@@ -368,7 +374,7 @@
     <t>0.0860</t>
   </si>
   <si>
-    <t>0.0838</t>
+    <t>0.0841</t>
   </si>
   <si>
     <t>0.2231</t>
@@ -377,10 +383,10 @@
     <t>0.5577 to 0.8947</t>
   </si>
   <si>
-    <t>0.5622 to 0.8906</t>
+    <t>0.5687 to 0.8986</t>
   </si>
   <si>
-    <t>-0.8244 to 0.0500</t>
+    <t>-0.8175 to 0.0572</t>
   </si>
 </sst>
 </file>
@@ -22012,7 +22018,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="533" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J2" s="597" t="s">
         <v>1</v>
@@ -22041,13 +22047,13 @@
         <v>55</v>
       </c>
       <c r="H3" s="587" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I3" s="542" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J3" s="598" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4">
@@ -22070,16 +22076,16 @@
         <v>46</v>
       </c>
       <c r="G4" s="441" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="H4" s="588" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I4" s="443" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J4" s="599" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -22105,13 +22111,13 @@
         <v>47</v>
       </c>
       <c r="H5" s="589" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I5" s="451" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J5" s="600" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6">
@@ -22134,16 +22140,16 @@
         <v>48</v>
       </c>
       <c r="G6" s="457" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H6" s="590" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I6" s="459" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J6" s="601" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7">
@@ -22166,16 +22172,16 @@
         <v>49</v>
       </c>
       <c r="G7" s="465" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H7" s="591" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I7" s="467" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J7" s="602" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8">
@@ -22198,16 +22204,16 @@
         <v>50</v>
       </c>
       <c r="G8" s="473" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H8" s="592" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I8" s="475" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J8" s="603" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
@@ -22230,16 +22236,16 @@
         <v>51</v>
       </c>
       <c r="G9" s="481" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H9" s="593" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I9" s="483" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J9" s="604" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10">
@@ -22265,13 +22271,13 @@
         <v>52</v>
       </c>
       <c r="H10" s="594" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I10" s="491" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J10" s="605" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
@@ -22297,13 +22303,13 @@
         <v>53</v>
       </c>
       <c r="H11" s="595" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I11" s="499" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J11" s="606" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
@@ -22326,16 +22332,16 @@
         <v>54</v>
       </c>
       <c r="G12" s="549" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H12" s="596" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I12" s="551" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J12" s="607" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" s="637" customFormat="true" ht="38" customHeight="true">
@@ -22398,7 +22404,7 @@
   <sheetData>
     <row r="1" s="779" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="778" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B1" s="768" t="s">
         <v>1</v>
@@ -22430,7 +22436,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="884" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D2" s="885" t="s">
         <v>1</v>
@@ -22439,7 +22445,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="887" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="888" t="s">
         <v>1</v>
@@ -22456,22 +22462,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="891" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D3" s="892" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E3" s="915" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F3" s="894" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G3" s="895" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H3" s="925" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -22479,25 +22485,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="911" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" s="852" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D4" s="853" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E4" s="916" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F4" s="855" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G4" s="856" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H4" s="926" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
@@ -22505,25 +22511,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="912" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" s="858" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D5" s="859" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E5" s="917" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F5" s="861" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G5" s="862" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H5" s="927" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6">
@@ -22531,7 +22537,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="913" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C6" s="898" t="s">
         <v>1</v>
@@ -22540,7 +22546,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="918" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F6" s="901" t="s">
         <v>1</v>
@@ -22549,7 +22555,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="928" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" s="952" customFormat="true" ht="38" customHeight="true">
@@ -22557,7 +22563,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="951" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C7" s="944" t="s">
         <v>1</v>
@@ -22602,7 +22608,7 @@
   <sheetData>
     <row r="1" s="1124" customFormat="true" ht="30" customHeight="true">
       <c r="A1" s="1123" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1116" t="s">
         <v>1</v>
@@ -22625,7 +22631,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1258" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D2" s="1259" t="s">
         <v>1</v>
@@ -22639,16 +22645,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="1283" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C3" s="1262" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D3" s="1263" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E3" s="1309" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
@@ -22656,16 +22662,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="1284" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C4" s="1207" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D4" s="1208" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E4" s="1310" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5">
@@ -22673,16 +22679,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="1285" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C5" s="1210" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D5" s="1211" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E5" s="1311" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6">
@@ -22690,16 +22696,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="1286" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C6" s="1213" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D6" s="1214" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E6" s="1312" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -22710,7 +22716,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="1247" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D7" s="1248" t="s">
         <v>1</v>
@@ -22724,10 +22730,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="1288" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C8" s="1219" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D8" s="1220" t="s">
         <v>1</v>
@@ -22741,10 +22747,10 @@
         <v>1</v>
       </c>
       <c r="B9" s="1289" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C9" s="1222" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D9" s="1223" t="s">
         <v>1</v>
@@ -22758,10 +22764,10 @@
         <v>1</v>
       </c>
       <c r="B10" s="1290" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C10" s="1225" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D10" s="1226" t="s">
         <v>1</v>
@@ -22775,10 +22781,10 @@
         <v>1</v>
       </c>
       <c r="B11" s="1291" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C11" s="1228" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D11" s="1229" t="s">
         <v>1</v>
@@ -22792,10 +22798,10 @@
         <v>1</v>
       </c>
       <c r="B12" s="1292" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C12" s="1231" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D12" s="1232" t="s">
         <v>1</v>
@@ -22809,10 +22815,10 @@
         <v>1</v>
       </c>
       <c r="B13" s="1293" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C13" s="1234" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D13" s="1235" t="s">
         <v>1</v>
@@ -22826,10 +22832,10 @@
         <v>1</v>
       </c>
       <c r="B14" s="1294" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="1266" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D14" s="1267" t="s">
         <v>1</v>
@@ -22843,7 +22849,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="1334" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" s="1330" t="s">
         <v>1</v>

</xml_diff>